<commit_message>
chore: working on slides
</commit_message>
<xml_diff>
--- a/program.xlsx
+++ b/program.xlsx
@@ -5,16 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveunibo-my.sharepoint.com/personal/matteo_francia2_studio_unibo_it/Documents/teaching-bigdata/AA2526-unibo-mldm/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\repos\teaching\AA2627-unibo-mldm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="224" documentId="11_F25DC773A252ABDACC10480B991D78805BDE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{008EF8F6-9F71-4F2A-8B12-D734D1DE2C08}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4191F236-78AA-48EE-BFD7-F900160C04C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="15990" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7848" yWindow="6408" windowWidth="34560" windowHeight="18600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="AA2526" sheetId="2" r:id="rId1"/>
-    <sheet name="AA2425" sheetId="1" r:id="rId2"/>
+    <sheet name="AA2627" sheetId="3" r:id="rId1"/>
+    <sheet name="AA2526" sheetId="2" r:id="rId2"/>
+    <sheet name="AA2425" sheetId="1" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="55">
   <si>
     <t>When</t>
   </si>
@@ -161,6 +162,48 @@
   </si>
   <si>
     <t>Lab: Challenge Solution + AutoML</t>
+  </si>
+  <si>
+    <t>LAB. 3.3 (9-12)</t>
+  </si>
+  <si>
+    <t>LAB. 3.3 (14-17)</t>
+  </si>
+  <si>
+    <t>AULA 2.4 (9-11)</t>
+  </si>
+  <si>
+    <t>AULA 3.7 (14-16)</t>
+  </si>
+  <si>
+    <t>Intro + 01-ML</t>
+  </si>
+  <si>
+    <t>02-DT</t>
+  </si>
+  <si>
+    <t>Summing UP</t>
+  </si>
+  <si>
+    <t>Lab-Classification</t>
+  </si>
+  <si>
+    <t>05-NN</t>
+  </si>
+  <si>
+    <t>02-DT + 03-KNN</t>
+  </si>
+  <si>
+    <t>Clustering</t>
+  </si>
+  <si>
+    <t>Association Rules</t>
+  </si>
+  <si>
+    <t>HPO</t>
+  </si>
+  <si>
+    <t>Anomaly</t>
   </si>
 </sst>
 </file>
@@ -237,7 +280,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -282,6 +325,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -562,22 +608,513 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D74ABA20-3F0C-49B2-9D00-1BC45AE4AF02}">
+  <dimension ref="A1:H20"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.21875" customWidth="1"/>
+    <col min="4" max="4" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="38.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="12">
+        <v>46279</v>
+      </c>
+      <c r="B2" s="5">
+        <f>WEEKDAY(A2)-1</f>
+        <v>1</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" t="s">
+        <v>45</v>
+      </c>
+      <c r="G2" s="7">
+        <v>3</v>
+      </c>
+      <c r="H2" s="16">
+        <f>SUM($G$2:G2)/$G$20</f>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="12">
+        <v>46280</v>
+      </c>
+      <c r="B3" s="5">
+        <f t="shared" ref="B3:B17" si="0">WEEKDAY(A3)-1</f>
+        <v>2</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G3" s="7">
+        <v>2</v>
+      </c>
+      <c r="H3" s="16">
+        <f>SUM($G$2:G3)/$G$20</f>
+        <v>0.16666666666666666</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="12">
+        <v>46280</v>
+      </c>
+      <c r="B4" s="5">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" t="s">
+        <v>50</v>
+      </c>
+      <c r="G4" s="7">
+        <v>3</v>
+      </c>
+      <c r="H4" s="16">
+        <f>SUM($G$2:G4)/$G$20</f>
+        <v>0.26666666666666666</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="12">
+        <v>46281</v>
+      </c>
+      <c r="B5" s="5">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G5" s="7">
+        <v>2</v>
+      </c>
+      <c r="H5" s="16">
+        <f>SUM($G$2:G5)/$G$20</f>
+        <v>0.33333333333333331</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="12">
+        <f>A2+7</f>
+        <v>46286</v>
+      </c>
+      <c r="B6" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="G6" s="7">
+        <v>3</v>
+      </c>
+      <c r="H6" s="16">
+        <f>SUM($G$2:G6)/$G$20</f>
+        <v>0.43333333333333335</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="12">
+        <f t="shared" ref="A7:A17" si="1">A3+7</f>
+        <v>46287</v>
+      </c>
+      <c r="B7" s="5">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" t="s">
+        <v>51</v>
+      </c>
+      <c r="G7" s="7">
+        <v>2</v>
+      </c>
+      <c r="H7" s="16">
+        <f>SUM($G$2:G7)/$G$20</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="12">
+        <f t="shared" si="1"/>
+        <v>46287</v>
+      </c>
+      <c r="B8" s="5">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" t="s">
+        <v>51</v>
+      </c>
+      <c r="G8" s="7">
+        <v>3</v>
+      </c>
+      <c r="H8" s="16">
+        <f>SUM($G$2:G8)/$G$20</f>
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="12">
+        <f t="shared" si="1"/>
+        <v>46288</v>
+      </c>
+      <c r="B9" s="5">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="G9" s="7">
+        <v>2</v>
+      </c>
+      <c r="H9" s="16">
+        <f>SUM($G$2:G9)/$G$20</f>
+        <v>0.66666666666666663</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="12">
+        <f t="shared" si="1"/>
+        <v>46293</v>
+      </c>
+      <c r="B10" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C10" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="H10" s="16">
+        <f>SUM($G$2:G10)/$G$20</f>
+        <v>0.66666666666666663</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="12">
+        <f t="shared" si="1"/>
+        <v>46294</v>
+      </c>
+      <c r="B11" s="5">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="H11" s="16">
+        <f>SUM($G$2:G11)/$G$20</f>
+        <v>0.66666666666666663</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" s="12">
+        <f t="shared" si="1"/>
+        <v>46294</v>
+      </c>
+      <c r="B12" s="5">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="H12" s="16">
+        <f>SUM($G$2:G12)/$G$20</f>
+        <v>0.66666666666666663</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" s="12">
+        <f t="shared" si="1"/>
+        <v>46295</v>
+      </c>
+      <c r="B13" s="5">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="H13" s="16">
+        <f>SUM($G$2:G13)/$G$20</f>
+        <v>0.66666666666666663</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" s="12">
+        <f t="shared" si="1"/>
+        <v>46300</v>
+      </c>
+      <c r="B14" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E14" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="G14" s="7">
+        <v>3</v>
+      </c>
+      <c r="H14" s="16">
+        <f>SUM($G$2:G14)/$G$20</f>
+        <v>0.76666666666666672</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" s="12">
+        <f t="shared" si="1"/>
+        <v>46301</v>
+      </c>
+      <c r="B15" s="5">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E15" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="G15" s="7">
+        <v>2</v>
+      </c>
+      <c r="H15" s="16">
+        <f>SUM($G$2:G15)/$G$20</f>
+        <v>0.83333333333333337</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" s="12">
+        <f t="shared" si="1"/>
+        <v>46301</v>
+      </c>
+      <c r="B16" s="5">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E16" t="s">
+        <v>53</v>
+      </c>
+      <c r="G16" s="7">
+        <v>3</v>
+      </c>
+      <c r="H16" s="16">
+        <f>SUM($G$2:G16)/$G$20</f>
+        <v>0.93333333333333335</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" s="12">
+        <f t="shared" si="1"/>
+        <v>46302</v>
+      </c>
+      <c r="B17" s="5">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E17" t="s">
+        <v>47</v>
+      </c>
+      <c r="G17" s="7">
+        <v>2</v>
+      </c>
+      <c r="H17" s="16">
+        <f>SUM($G$2:G17)/$G$20</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H18" s="16"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E19" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="G19" s="5">
+        <f>SUM(G2:G17)</f>
+        <v>30</v>
+      </c>
+      <c r="H19" s="4"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E20" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="G20" s="1">
+        <v>30</v>
+      </c>
+      <c r="H20" s="1"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A2:A17">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E1BA7BF-4F83-4B95-BD26-B9FD6BCF8777}">
   <dimension ref="A1:I17"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.26953125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="13.26953125" style="14" customWidth="1"/>
-    <col min="4" max="4" width="6.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="39.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.26953125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="8.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.21875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="13.21875" style="14" customWidth="1"/>
+    <col min="4" max="4" width="6.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="39.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.21875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="8.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.21875" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -604,7 +1141,7 @@
       </c>
       <c r="I1" s="3"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="12">
         <v>45924</v>
       </c>
@@ -632,13 +1169,13 @@
         <v>8.3333333333333329E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="12">
         <f>A2+7</f>
         <v>45931</v>
       </c>
       <c r="B3" s="5">
-        <f t="shared" ref="B3:B15" si="0">WEEKDAY(A3)-1</f>
+        <f t="shared" ref="B3:B14" si="0">WEEKDAY(A3)-1</f>
         <v>3</v>
       </c>
       <c r="C3" s="10" t="s">
@@ -661,9 +1198,9 @@
         <v>0.16666666666666666</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
-        <f t="shared" ref="A4:A15" si="1">A3+7</f>
+        <f t="shared" ref="A4:A14" si="1">A3+7</f>
         <v>45938</v>
       </c>
       <c r="B4" s="5">
@@ -690,7 +1227,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <f t="shared" si="1"/>
         <v>45945</v>
@@ -716,7 +1253,7 @@
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="12">
         <f t="shared" si="1"/>
         <v>45952</v>
@@ -742,7 +1279,7 @@
         <v>0.41666666666666669</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
         <f t="shared" si="1"/>
         <v>45959</v>
@@ -771,7 +1308,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="12">
         <f t="shared" si="1"/>
         <v>45966</v>
@@ -797,7 +1334,7 @@
         <v>0.58333333333333337</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="12">
         <f t="shared" si="1"/>
         <v>45973</v>
@@ -823,7 +1360,7 @@
         <v>0.66666666666666663</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="12">
         <f t="shared" si="1"/>
         <v>45980</v>
@@ -849,7 +1386,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="12">
         <f t="shared" si="1"/>
         <v>45987</v>
@@ -875,7 +1412,7 @@
         <v>0.83333333333333337</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="12">
         <f t="shared" si="1"/>
         <v>45994</v>
@@ -901,7 +1438,7 @@
         <v>0.91666666666666663</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="12">
         <f>A12+7</f>
         <v>46001</v>
@@ -927,7 +1464,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="12">
         <f t="shared" si="1"/>
         <v>46008</v>
@@ -948,7 +1485,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="12"/>
       <c r="B15" s="5"/>
       <c r="C15" s="10"/>
@@ -961,7 +1498,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="12"/>
       <c r="B16" s="6"/>
       <c r="C16" s="13"/>
@@ -975,7 +1512,7 @@
       </c>
       <c r="H16" s="4"/>
     </row>
-    <row r="17" spans="5:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="5:7" x14ac:dyDescent="0.3">
       <c r="E17" s="9" t="s">
         <v>30</v>
       </c>
@@ -1001,23 +1538,23 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I17"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.81640625" customWidth="1"/>
-    <col min="2" max="2" width="4.26953125" style="1" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="13.26953125" style="14" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.77734375" customWidth="1"/>
+    <col min="2" max="2" width="4.21875" style="1" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="13.21875" style="14" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.21875" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1044,7 +1581,7 @@
       </c>
       <c r="I1" s="3"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="12">
         <v>45559</v>
       </c>
@@ -1072,7 +1609,7 @@
         <v>8.3333333333333329E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="12">
         <f>A2+7</f>
         <v>45566</v>
@@ -1101,7 +1638,7 @@
         <v>0.16666666666666666</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <f t="shared" ref="A4:A15" si="1">A3+7</f>
         <v>45573</v>
@@ -1127,7 +1664,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <f t="shared" si="1"/>
         <v>45580</v>
@@ -1153,7 +1690,7 @@
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="12">
         <f t="shared" si="1"/>
         <v>45587</v>
@@ -1179,7 +1716,7 @@
         <v>0.41666666666666669</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
         <f t="shared" si="1"/>
         <v>45594</v>
@@ -1205,7 +1742,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="8" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="12">
         <f t="shared" si="1"/>
         <v>45601</v>
@@ -1231,7 +1768,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="12">
         <f t="shared" si="1"/>
         <v>45608</v>
@@ -1257,7 +1794,7 @@
         <v>0.58333333333333337</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="12">
         <f t="shared" si="1"/>
         <v>45615</v>
@@ -1283,7 +1820,7 @@
         <v>0.66666666666666663</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="12">
         <f t="shared" si="1"/>
         <v>45622</v>
@@ -1309,7 +1846,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="12">
         <f t="shared" si="1"/>
         <v>45629</v>
@@ -1335,7 +1872,7 @@
         <v>0.83333333333333337</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="12">
         <f>A12+7</f>
         <v>45636</v>
@@ -1361,7 +1898,7 @@
         <v>0.91666666666666663</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="12">
         <f t="shared" si="1"/>
         <v>45643</v>
@@ -1387,7 +1924,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="12">
         <f t="shared" si="1"/>
         <v>45650</v>
@@ -1406,7 +1943,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="12"/>
       <c r="B16" s="6"/>
       <c r="C16" s="13"/>
@@ -1420,7 +1957,7 @@
       </c>
       <c r="H16" s="4"/>
     </row>
-    <row r="17" spans="5:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="5:7" x14ac:dyDescent="0.3">
       <c r="E17" s="9" t="s">
         <v>30</v>
       </c>

</xml_diff>